<commit_message>
se realizó ejercido pagado recaudado y recaudado de préstamos con renovación
</commit_message>
<xml_diff>
--- a/public/Guia/7000-Ejercido-Pagado-Recaudado-Renovacion-CuentasConceptos.xlsx
+++ b/public/Guia/7000-Ejercido-Pagado-Recaudado-Renovacion-CuentasConceptos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\Guia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\Guia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C18C44-54E0-499E-AB84-35E2A38EA95C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03F0EC16-D103-4CB9-8083-9DDBF039F6A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="30">
   <si>
     <t>cuenta</t>
   </si>
@@ -120,6 +120,12 @@
   </si>
   <si>
     <t>8.1.5.4.1.7.1.02.04</t>
+  </si>
+  <si>
+    <t>1.1.2.6.02.01</t>
+  </si>
+  <si>
+    <t>1.2.2.4.02.03</t>
   </si>
 </sst>
 </file>
@@ -536,8 +542,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="107.5703125" customWidth="1"/>
-    <col min="3" max="3" width="197" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="190" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -864,12 +870,32 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="C24" s="2"/>
+      <c r="A24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="C25" s="2"/>
+      <c r="A25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>

</xml_diff>